<commit_message>
Add project benchmarks and validation
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -487,7 +487,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.bajajauto.com</t>
+          <t>https://www.bajajfinserv.in</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -497,7 +497,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>customerservice@bajajauto.co.in</t>
+          <t>Akurdi, Pune, Maharashtra, India (registered office; verify on site)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -507,7 +507,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Emails: corporatesales@bajajauto.co.in; customerservice@bajajauto.co.in; deepti.singh@pitchforkpartners.com; ivana.edwards@pitchforkpartners.com | Phones: +91 7219821111; +912027406000; +912027407000; +912027472851</t>
+          <t>No direct contacts published (contact form only)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -517,7 +517,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>possible_parent_employee_count</t>
+          <t>incomplete_address,possible_parent_employee_count</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.hdfc.bank.in</t>
+          <t>https://www.hdfcergo.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Add/Modify Nominee</t>
+          <t>HDFC ERGO General Insurance Registered &amp; Corporate Office: 6th Floor, Leela Business Park, Andheri-Kurla Road, Andheri (East), Mumbai – 400 059</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Phones: 18001600</t>
+          <t>Emails: care@hdfcergo.com; healthclaims@hdfcergo.com; medical.services@allianz.com; travelclaims@hdfcergo.com | Phones: +91 022 6158 2020*; 0120-6234-6234; 0120-6740895*; 022 6158 2020</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.astrologyanswers.com</t>
+          <t>https://www.apollohospitals.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>101 Convention Center Dr STE 400, Las Vegas, Nevada, 89109, US</t>
+          <t>No. 21, Greams Lane, Off Greams Road, Chennai 600006, Tamil Nadu, India</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No direct contacts published (contact form only)</t>
+          <t>Phones: +1066; +91 4043441066; +914043441066; 08069991061</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.paisabazaar.com</t>
+          <t>https://www.drreddys.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ed effectively. His communication skills, positive attitude, and dedication towards his responsibilities truly reflect his commitment to the</t>
+          <t>8-2-337, Road No. 3, Banjara Hills, Hyderabad 500034, Telangana, India</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Emails: care@paisabazaar.com; creditreport@paisabazaar.com; escalationdesk@paisabazaar.com; mutualfunds@paisabazaar.com; npsgrievanceofficer@paisabazaar.com; servicehead@paisabazaar.com; stepupcare@paisabazaar.com | Phones: 18002088877; 18002585616; 18005703888</t>
+          <t>Phones: 040 4900 2900</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://web.whatsapp.com</t>
+          <t>https://www.manappuram.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -685,7 +685,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Manappuram House, Valapad, Thrissur, Kerala 680567, India</t>
+          <t>Office Manappuram Finance Limited, W - 4/ 638 A Manappuram House, P.O. Valapad,Thrissur, Kerala, India - 680 567</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>No direct contacts published (contact form only)</t>
+          <t>Phones: 1800-420-22-33</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.icici.bank.in</t>
+          <t>https://www.icicilombard.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ICICI Bank Towers, Bandra Kurla Complex, Mumbai, Maharashtra, 400051, IN</t>
+          <t>ICICI Lombard House, 414, Veer Savarkar Marg, Prabhadevi, Mumbai 400025, India</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -742,12 +742,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Phones: 1800%201080; 18001080; tel:1800%201080</t>
+          <t>No direct contacts published (contact form only)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>live+seed</t>
+          <t>seed</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://totalfucktube.com</t>
+          <t>https://www.maxhealthcare.in</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>live+seed</t>
+          <t>seed</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>live+seed</t>
+          <t>seed</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">

</xml_diff>